<commit_message>
scan: seg6 2026-07-22 17:29 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-22.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-22.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O125"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2594,21 +2594,21 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6741</v>
+        <v>6683</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>雍智科技</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>390.967311869736</v>
+        <v>393.4075687504804</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>57.6</v>
+        <v>1220</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,49 +2619,49 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>40.74292996178488</v>
+        <v>34.91133460620696</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>24.26550473228687</v>
+        <v>19.89590059423068</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.9566666701083192</v>
+        <v>0.4096194115258552</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M41" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.2680374288757734</v>
+        <v>-57.81851838607541</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6654</v>
+        <v>6741</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>天正國際</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>380.2045432332793</v>
+        <v>390.967311869736</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>179</v>
+        <v>57.6</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>48.75368402674627</v>
+        <v>40.74292996178488</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>30.39091254158249</v>
+        <v>24.26550473228687</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.1897209958435965</v>
+        <v>0.9566666701083192</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-3.766792346224417</v>
+        <v>-0.2680374288757734</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6743</v>
+        <v>6654</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>安普新</t>
+          <t>天正國際</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>379.5450684741928</v>
+        <v>380.2045432332793</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>30.05</v>
+        <v>179</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>49.14880146612923</v>
+        <v>48.75368402674627</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>32.1043093442286</v>
+        <v>30.39091254158249</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.4089534534564573</v>
+        <v>0.1897209958435965</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.1534632297822443</v>
+        <v>-3.766792346224417</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6715</v>
+        <v>6743</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>安普新</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>378.3880459396071</v>
+        <v>379.5450684741928</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>387</v>
+        <v>30.05</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>43.63563192329872</v>
+        <v>49.14880146612923</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>12.50119990244833</v>
+        <v>32.1043093442286</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>2.502061025108078</v>
+        <v>0.4089534534564573</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-4.991309956576936</v>
+        <v>-0.1534632297822443</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6651</v>
+        <v>6715</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>全宇昕</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>371.5274987866039</v>
+        <v>378.3880459396071</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>124</v>
+        <v>387</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>40.23196147568702</v>
+        <v>43.63563192329872</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>25.38999398688829</v>
+        <v>12.50119990244833</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.4071685530912531</v>
+        <v>2.502061025108078</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-4.692138490271445</v>
+        <v>-4.991309956576936</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6757</v>
+        <v>6651</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>台灣虎航-創</t>
+          <t>全宇昕</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>369.6924072190709</v>
+        <v>371.5274987866039</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>56.9</v>
+        <v>124</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>45.44915937061652</v>
+        <v>40.23196147568702</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>21.94011206734094</v>
+        <v>25.38999398688829</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.7175552495454603</v>
+        <v>0.4071685530912531</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.5196224414034307</v>
+        <v>-4.692138490271445</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6830</v>
+        <v>6757</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>汎銓</t>
+          <t>台灣虎航-創</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>365.9918877183337</v>
+        <v>369.6924072190709</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>370.5</v>
+        <v>56.9</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>33.67254367136107</v>
+        <v>45.44915937061652</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>32.83655078721413</v>
+        <v>21.94011206734094</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1.028512237359205</v>
+        <v>0.7175552495454603</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.2211237426069559</v>
+        <v>-0.5196224414034307</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6577</v>
+        <v>6830</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>勁豐</t>
+          <t>汎銓</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>359.323624195574</v>
+        <v>365.9918877183337</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>78.09999999999999</v>
+        <v>370.5</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>53.73217920119809</v>
+        <v>33.67254367136107</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>18.33909648706926</v>
+        <v>32.83655078721413</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.123255784426171</v>
+        <v>1.028512237359205</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.1469591758720642</v>
+        <v>-0.2211237426069559</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6515</v>
+        <v>6577</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>勁豐</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>356.8377282375014</v>
+        <v>359.323624195574</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>6500</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>36.7258978464067</v>
+        <v>53.73217920119809</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>22.84423179042504</v>
+        <v>18.33909648706926</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.383772823750138</v>
+        <v>1.123255784426171</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-172.3585311987679</v>
+        <v>0.1469591758720642</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6782</v>
+        <v>6515</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>視陽</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>356.1189101130389</v>
+        <v>356.8377282375014</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>188.5</v>
+        <v>6500</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>38.80187109631298</v>
+        <v>36.7258978464067</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>15.80492434684025</v>
+        <v>22.84423179042504</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.9238626554422908</v>
+        <v>1.383772823750138</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.496407880455064</v>
+        <v>-172.3585311987679</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6680</v>
+        <v>6782</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>鑫創電子</t>
+          <t>視陽</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>353.775870104671</v>
+        <v>356.1189101130389</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>56</v>
+        <v>188.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>54.21097466331045</v>
+        <v>38.80187109631298</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>6.828920908470794</v>
+        <v>15.80492434684025</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.618840335361648</v>
+        <v>0.9238626554422908</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.6551843409406926</v>
+        <v>-1.496407880455064</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6645</v>
+        <v>6680</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>金萬林-創</t>
+          <t>鑫創電子</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>353.4815853990139</v>
+        <v>353.775870104671</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>13.35</v>
+        <v>56</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>35.76077836763577</v>
+        <v>54.21097466331045</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>33.10204231947253</v>
+        <v>6.828920908470794</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.7370799759939856</v>
+        <v>0.618840335361648</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.3760258734001226</v>
+        <v>0.6551843409406926</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6606</v>
+        <v>6645</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>建德工業</t>
+          <t>金萬林-創</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>352.2929018091982</v>
+        <v>353.4815853990139</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>25.7</v>
+        <v>13.35</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>55.60388018737423</v>
+        <v>35.76077836763577</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>16.01346182994123</v>
+        <v>33.10204231947253</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.4798890122905605</v>
+        <v>0.7370799759939856</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0843506365409027</v>
+        <v>-0.3760258734001226</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6840</v>
+        <v>6606</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>建德工業</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>349.3832328795395</v>
+        <v>352.2929018091982</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>60.7</v>
+        <v>25.7</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>41.31474179177603</v>
+        <v>55.60388018737423</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>11.72315786960568</v>
+        <v>16.01346182994123</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.5296607959929889</v>
+        <v>0.4798890122905605</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.3549977260582087</v>
+        <v>0.0843506365409027</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6670</v>
+        <v>6840</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>復盛應用</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>347.7831538786571</v>
+        <v>349.3832328795395</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>262.5</v>
+        <v>60.7</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>49.55824882770564</v>
+        <v>41.31474179177603</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>12.0845902242996</v>
+        <v>11.72315786960568</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.7422743975142315</v>
+        <v>0.5296607959929889</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.6724083528871008</v>
+        <v>-0.3549977260582087</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6684</v>
+        <v>6670</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>安格</t>
+          <t>復盛應用</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>346.1187649294412</v>
+        <v>347.7831538786571</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>49.95</v>
+        <v>262.5</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>43.31667888668766</v>
+        <v>49.55824882770564</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>21.85564514655065</v>
+        <v>12.0845902242996</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.1323848856405159</v>
+        <v>0.7422743975142315</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-1.114849669438796</v>
+        <v>0.6724083528871008</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6805</v>
+        <v>6684</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>安格</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>345.9390170210808</v>
+        <v>346.1187649294412</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>1395</v>
+        <v>49.95</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>39.89792159494299</v>
+        <v>43.31667888668766</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>34.29603544114862</v>
+        <v>21.85564514655065</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.5276035677651211</v>
+        <v>0.1323848856405159</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-3.561600725394428</v>
+        <v>-1.114849669438796</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6756</v>
+        <v>6805</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>342.9460469493617</v>
+        <v>345.9390170210808</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>95.8</v>
+        <v>1395</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>47.80533247865024</v>
+        <v>39.89792159494299</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>18.83816433288217</v>
+        <v>34.29603544114862</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.6867365749405353</v>
+        <v>0.5276035677651211</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.7286607715424229</v>
+        <v>-3.561600725394428</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6763</v>
+        <v>6756</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>341.1924651710983</v>
+        <v>342.9460469493617</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>42.9</v>
+        <v>95.8</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>38.06288778530104</v>
+        <v>47.80533247865024</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>25.60954668406644</v>
+        <v>18.83816433288217</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.5168093481279182</v>
+        <v>0.6867365749405353</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.3381075812855626</v>
+        <v>-0.7286607715424229</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6664</v>
+        <v>6763</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>群翊</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>337.021988498829</v>
+        <v>341.1924651710983</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>371</v>
+        <v>42.9</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>45.76122596301554</v>
+        <v>38.06288778530104</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>21.05600478189636</v>
+        <v>25.60954668406644</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.5483577703514744</v>
+        <v>0.5168093481279182</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-1.198424215372079</v>
+        <v>-0.3381075812855626</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6761</v>
+        <v>6664</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>群翊</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>336.4175305546187</v>
+        <v>337.021988498829</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>155.5</v>
+        <v>371</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>34.07455530428643</v>
+        <v>45.76122596301554</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>21.03838862977456</v>
+        <v>21.05600478189636</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.4365362662600198</v>
+        <v>0.5483577703514744</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-3.048950132051824</v>
+        <v>-1.198424215372079</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3707,21 +3707,21 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6498</v>
+        <v>6761</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>334.4734660177384</v>
+        <v>336.4175305546187</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>81.90000000000001</v>
+        <v>155.5</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>33.45792434864846</v>
+        <v>34.07455530428643</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>29.05149313242534</v>
+        <v>21.03838862977456</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.2773232685105061</v>
+        <v>0.4365362662600198</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.9156031894862586</v>
+        <v>-3.048950132051824</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6494</v>
+        <v>6498</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>九齊</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>333.5127801471885</v>
+        <v>334.4734660177384</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>51</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>32.35395733963146</v>
+        <v>33.45792434864846</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>29.27092170885568</v>
+        <v>29.05149313242534</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.2872707839282326</v>
+        <v>0.2773232685105061</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.012568194787573</v>
+        <v>-0.9156031894862586</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6788</v>
+        <v>6494</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>九齊</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>332.7994709499725</v>
+        <v>333.5127801471885</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>354.5</v>
+        <v>51</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>35.61369062708422</v>
+        <v>32.35395733963146</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>23.71536036593079</v>
+        <v>29.27092170885568</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.3828715365239294</v>
+        <v>0.2872707839282326</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-7.307943123683245</v>
+        <v>-2.012568194787573</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6561</v>
+        <v>6788</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>331.9197911559826</v>
+        <v>332.7994709499725</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>328</v>
+        <v>354.5</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.20023503515865</v>
+        <v>35.61369062708422</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>25.83782286435604</v>
+        <v>23.71536036593079</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.2178277438336387</v>
+        <v>0.3828715365239294</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.1304526770036851</v>
+        <v>-7.307943123683245</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6799</v>
+        <v>6561</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>來頡</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>330.0566884944859</v>
+        <v>331.9197911559826</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>84.8</v>
+        <v>328</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>39.20136784096192</v>
+        <v>45.20023503515865</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>22.69794444997337</v>
+        <v>25.83782286435604</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.3782651950963491</v>
+        <v>0.2178277438336387</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-2.037123168180344</v>
+        <v>-0.1304526770036851</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6671</v>
+        <v>6799</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>三能-KY</t>
+          <t>來頡</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>323.7168272845328</v>
+        <v>330.0566884944859</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>24</v>
+        <v>84.8</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>29.55533889895621</v>
+        <v>39.20136784096192</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>23.43682398102342</v>
+        <v>22.69794444997337</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>1.996395811761488</v>
+        <v>0.3782651950963491</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.07355217581747529</v>
+        <v>-2.037123168180344</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6658</v>
+        <v>6671</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>聯策</t>
+          <t>三能-KY</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>322.6107753970732</v>
+        <v>323.7168272845328</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>162.5</v>
+        <v>24</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>39.39318649354311</v>
+        <v>29.55533889895621</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>22.88004187666476</v>
+        <v>23.43682398102342</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.4198166314036394</v>
+        <v>1.996395811761488</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-5.504713283725975</v>
+        <v>0.07355217581747529</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6691</v>
+        <v>6658</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>洋基工程</t>
+          <t>聯策</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>320.9148117045913</v>
+        <v>322.6107753970732</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>726</v>
+        <v>162.5</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>51.32829470442447</v>
+        <v>39.39318649354311</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>17.47241781977504</v>
+        <v>22.88004187666476</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.4720643462045285</v>
+        <v>0.4198166314036394</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-6.168687993547108</v>
+        <v>-5.504713283725975</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6706</v>
+        <v>6691</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>洋基工程</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>316.7596323085647</v>
+        <v>320.9148117045913</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>116.5</v>
+        <v>726</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>34.41585089723726</v>
+        <v>51.32829470442447</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>28.0296480119088</v>
+        <v>17.47241781977504</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1.093514773916151</v>
+        <v>0.4720643462045285</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-2.215079193557582</v>
+        <v>-6.168687993547108</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6556</v>
+        <v>6706</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>316.2504304691074</v>
+        <v>316.7596323085647</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>64.2</v>
+        <v>116.5</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>25.49075376054061</v>
+        <v>34.41585089723726</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>31.06627544318166</v>
+        <v>28.0296480119088</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1.477536983873289</v>
+        <v>1.093514773916151</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.7092433566811478</v>
+        <v>-2.215079193557582</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6754</v>
+        <v>6556</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>309.3448904451045</v>
+        <v>316.2504304691074</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>42.15</v>
+        <v>64.2</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>40.73544605626647</v>
+        <v>25.49075376054061</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>12.89100442556569</v>
+        <v>31.06627544318166</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.5886916427450375</v>
+        <v>1.477536983873289</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0571451712533943</v>
+        <v>-0.7092433566811478</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6838</v>
+        <v>6754</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>309.2599643792602</v>
+        <v>309.3448904451045</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>23.85</v>
+        <v>42.15</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>46.17624799593639</v>
+        <v>40.73544605626647</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>10.35161332313681</v>
+        <v>12.89100442556569</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.7924031081205996</v>
+        <v>0.5886916427450375</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0069082877132225</v>
+        <v>-0.0571451712533943</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6742</v>
+        <v>6838</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>澤米</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>305.9197619736573</v>
+        <v>309.2599643792602</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>44.85</v>
+        <v>23.85</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>28.60241246165834</v>
+        <v>46.17624799593639</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>22.95639714200087</v>
+        <v>10.35161332313681</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.2563970883431348</v>
+        <v>0.7924031081205996</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-2.188971732331881</v>
+        <v>0.0069082877132225</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6821</v>
+        <v>6742</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>聯寶</t>
+          <t>澤米</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>300.7334066556796</v>
+        <v>305.9197619736573</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>43.85</v>
+        <v>44.85</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>25.70164537905538</v>
+        <v>28.60241246165834</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>25.28330365101565</v>
+        <v>22.95639714200087</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.1447210313758186</v>
+        <v>0.2563970883431348</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-1.249392126390249</v>
+        <v>-2.188971732331881</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6735</v>
+        <v>6821</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>美達科技</t>
+          <t>聯寶</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>300.5487207603256</v>
+        <v>300.7334066556796</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>68.90000000000001</v>
+        <v>43.85</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>27.49437193364369</v>
+        <v>25.70164537905538</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>24.47714385096468</v>
+        <v>25.28330365101565</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.5547573852311681</v>
+        <v>0.1447210313758186</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.9766772215159856</v>
+        <v>-1.249392126390249</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4502,21 +4502,21 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6532</v>
+        <v>6735</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>美達科技</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>298.3502667928296</v>
+        <v>300.5487207603256</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>70.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>30.92671138384372</v>
+        <v>27.49437193364369</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>29.12661486535828</v>
+        <v>24.47714385096468</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.3811689489909101</v>
+        <v>0.5547573852311681</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-1.150331796024499</v>
+        <v>-0.9766772215159856</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4555,21 +4555,21 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6584</v>
+        <v>6532</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>297.8785933803841</v>
+        <v>298.3502667928296</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>552</v>
+        <v>70.3</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,49 +4580,49 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.65837449242306</v>
+        <v>30.92671138384372</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.38971198007451</v>
+        <v>29.12661486535828</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.4785902050088232</v>
+        <v>0.3811689489909101</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M78" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-17.20369138660319</v>
+        <v>-1.150331796024499</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6588</v>
+        <v>6584</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>294.9393204874674</v>
+        <v>297.8785933803841</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>73.59999999999999</v>
+        <v>552</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,49 +4633,49 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>33.12703341536896</v>
+        <v>35.65837449242306</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>29.57878766696684</v>
+        <v>18.38971198007451</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.790097275860573</v>
+        <v>0.4785902050088232</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M79" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.0031301523980022</v>
+        <v>-17.20369138660319</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6641</v>
+        <v>6588</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>290.9540047280858</v>
+        <v>294.9393204874674</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>17.95</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>44.70282765873229</v>
+        <v>33.12703341536896</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>15.16919013454516</v>
+        <v>29.57878766696684</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.9383066882150676</v>
+        <v>0.790097275860573</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.052033014051827</v>
+        <v>-0.0031301523980022</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6655</v>
+        <v>6641</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>科定</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>288.3830941063425</v>
+        <v>290.9540047280858</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>118</v>
+        <v>17.95</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>49.13938376339074</v>
+        <v>44.70282765873229</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>6.291698764296898</v>
+        <v>15.16919013454516</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.8074594974399734</v>
+        <v>0.9383066882150676</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.303300785076116</v>
+        <v>-0.052033014051827</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6790</v>
+        <v>6655</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>永豐實</t>
+          <t>科定</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>284.8302317995714</v>
+        <v>288.3830941063425</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>38.5</v>
+        <v>118</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>37.24845740945327</v>
+        <v>49.13938376339074</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>25.03124901809807</v>
+        <v>6.291698764296898</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.6872616355391238</v>
+        <v>0.8074594974399734</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.1661918026349292</v>
+        <v>0.303300785076116</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6546</v>
+        <v>6790</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>永豐實</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>280.2244149188991</v>
+        <v>284.8302317995714</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>60.8</v>
+        <v>38.5</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>35.05815032055263</v>
+        <v>37.24845740945327</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>25.03208133017244</v>
+        <v>25.03124901809807</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.6119873971569305</v>
+        <v>0.6872616355391238</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.8018461613633914</v>
+        <v>-0.1661918026349292</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6776</v>
+        <v>6546</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>276.2984525241172</v>
+        <v>280.2244149188991</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>55.1</v>
+        <v>60.8</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>46.26226265274916</v>
+        <v>35.05815032055263</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>16.61040355732558</v>
+        <v>25.03208133017244</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.5704215490640301</v>
+        <v>0.6119873971569305</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.135679862402947</v>
+        <v>-0.8018461613633914</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6643</v>
+        <v>6776</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>275.9731179271287</v>
+        <v>276.2984525241172</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>424</v>
+        <v>55.1</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>39.96026322901459</v>
+        <v>46.26226265274916</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>22.52139579619215</v>
+        <v>16.61040355732558</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5068914382215227</v>
+        <v>0.5704215490640301</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-1.169271136706417</v>
+        <v>0.135679862402947</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6792</v>
+        <v>6643</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>274.1270616597595</v>
+        <v>275.9731179271287</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>54.3</v>
+        <v>424</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,16 +5004,16 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>33.68404143208356</v>
+        <v>39.96026322901459</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>21.25432019806948</v>
+        <v>22.52139579619215</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.4133301883749435</v>
+        <v>0.5068914382215227</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.9259480197218766</v>
+        <v>-1.169271136706417</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6605</v>
+        <v>6792</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>271.1367405559721</v>
+        <v>274.1270616597595</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>135.5</v>
+        <v>54.3</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>52.59335178517178</v>
+        <v>33.68404143208356</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>15.62638036187575</v>
+        <v>21.25432019806948</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>1.212742415471408</v>
+        <v>0.4133301883749435</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.1079686456847426</v>
+        <v>-0.9259480197218766</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, liquidity_ok, hist_turn_positive</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6530</v>
+        <v>6727</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>亞泰金屬</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>270.2410612405651</v>
+        <v>272.2319039505276</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>72.90000000000001</v>
+        <v>365.5</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>33.34285734461285</v>
+        <v>40.82292610583688</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>31.47372603954212</v>
+        <v>15.93810237033229</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.5711125229073821</v>
+        <v>0.256051193818755</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.5994737488508539</v>
+        <v>-11.99767330473464</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6689</v>
+        <v>6605</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>266.5859815086105</v>
+        <v>271.1367405559721</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>62</v>
+        <v>135.5</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>41.58567123535015</v>
+        <v>52.59335178517178</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>20.23674510123255</v>
+        <v>15.62638036187575</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5555513381651426</v>
+        <v>1.212742415471408</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.052110399042218</v>
+        <v>0.1079686456847426</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, liquidity_ok, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6722</v>
+        <v>6530</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>266.3790393114803</v>
+        <v>270.2410612405651</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>34.85</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>45.88168337052116</v>
+        <v>33.34285734461285</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>39.57058519022977</v>
+        <v>31.47372603954212</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.7415378112782219</v>
+        <v>0.5711125229073821</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.120435046241955</v>
+        <v>-0.5994737488508539</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6789</v>
+        <v>6689</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>采鈺</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>264.8968819267619</v>
+        <v>266.5859815086105</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>492</v>
+        <v>62</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>46.96191493946127</v>
+        <v>41.58567123535015</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>12.09855063327187</v>
+        <v>20.23674510123255</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6773298604398558</v>
+        <v>0.5555513381651426</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-4.084647614868486</v>
+        <v>-0.052110399042218</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6526</v>
+        <v>6722</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>263.9086323875125</v>
+        <v>266.3790393114803</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>591</v>
+        <v>34.85</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.36767859146151</v>
+        <v>45.88168337052116</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>15.60749818619076</v>
+        <v>39.57058519022977</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4165306759806079</v>
+        <v>0.7415378112782219</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-10.98509491863872</v>
+        <v>0.120435046241955</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6486</v>
+        <v>6789</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>互動</t>
+          <t>采鈺</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>260.1200304391867</v>
+        <v>264.8968819267619</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>76.7</v>
+        <v>492</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>33.75950959415333</v>
+        <v>46.96191493946127</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>22.15938512066026</v>
+        <v>12.09855063327187</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5903626864134741</v>
+        <v>0.6773298604398558</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.7080965983887038</v>
+        <v>-4.084647614868486</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6624</v>
+        <v>6526</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>萬年清</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>259.939751732527</v>
+        <v>263.9086323875125</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0</v>
+        <v>591</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>30.38473420923914</v>
+        <v>41.36767859146151</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>8.700584725904857</v>
+        <v>15.60749818619076</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.0004007980334176</v>
+        <v>0.4165306759806079</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-2.482130061097782</v>
+        <v>-10.98509491863872</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6835</v>
+        <v>6486</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>互動</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>255.5369029357045</v>
+        <v>260.1200304391867</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>31.75</v>
+        <v>76.7</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>27.84199616779981</v>
+        <v>33.75950959415333</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>39.4449872549782</v>
+        <v>22.15938512066026</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.4971824517724126</v>
+        <v>0.5903626864134741</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.1975006589942931</v>
+        <v>-0.7080965983887038</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5509,21 +5509,21 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6582</v>
+        <v>6624</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>申豐</t>
+          <t>萬年清</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>251.35153228391</v>
+        <v>259.939751732527</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>32.25</v>
+        <v>0</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>48.38432953388097</v>
+        <v>30.38473420923914</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>27.18673814713156</v>
+        <v>8.700584725904857</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.2728722667934589</v>
+        <v>0.0004007980334176</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1265746186585008</v>
+        <v>-2.482130061097782</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6725</v>
+        <v>6835</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>矽科宏晟</t>
+          <t>圓裕</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>249.5848002550168</v>
+        <v>255.5369029357045</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>315</v>
+        <v>31.75</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>49.29832175637037</v>
+        <v>27.84199616779981</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>15.47949786775422</v>
+        <v>39.4449872549782</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.4849309676056608</v>
+        <v>0.4971824517724126</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-2.304441358543534</v>
+        <v>-0.1975006589942931</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6531</v>
+        <v>6582</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>申豐</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>248.5408152578883</v>
+        <v>251.35153228391</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>908</v>
+        <v>32.25</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>48.51857715707485</v>
+        <v>48.38432953388097</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>15.84818444704954</v>
+        <v>27.18673814713156</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.730474711181773</v>
+        <v>0.2728722667934589</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-8.077822819318065</v>
+        <v>-0.1265746186585008</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6560</v>
+        <v>6725</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>矽科宏晟</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>245.7187800488993</v>
+        <v>249.5848002550168</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>33.35</v>
+        <v>315</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>33.46467879155651</v>
+        <v>49.29832175637037</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>26.21494850313197</v>
+        <v>15.47949786775422</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.3732103185074037</v>
+        <v>0.4849309676056608</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.5345522700054772</v>
+        <v>-2.304441358543534</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6698</v>
+        <v>6531</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>238.9803067917359</v>
+        <v>248.5408152578883</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>35.15</v>
+        <v>908</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>37.08555171679339</v>
+        <v>48.51857715707485</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>21.29845242120722</v>
+        <v>15.84818444704954</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.4211547326288706</v>
+        <v>0.730474711181773</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.964676505925196</v>
+        <v>-8.077822819318065</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6794</v>
+        <v>6560</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>236.772490499828</v>
+        <v>245.7187800488993</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>77.90000000000001</v>
+        <v>33.35</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.44731251339184</v>
+        <v>33.46467879155651</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>15.04700803777743</v>
+        <v>26.21494850313197</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5944984271295312</v>
+        <v>0.3732103185074037</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.334065529109323</v>
+        <v>-0.5345522700054772</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6581</v>
+        <v>6698</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>232.4922194540182</v>
+        <v>238.9803067917359</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>107</v>
+        <v>35.15</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>46.37175414619171</v>
+        <v>37.08555171679339</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>8.967333247108776</v>
+        <v>21.29845242120722</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.388950364695412</v>
+        <v>0.4211547326288706</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0336541127624466</v>
+        <v>-0.964676505925196</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6558</v>
+        <v>6794</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>226.1876616354878</v>
+        <v>236.772490499828</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>27.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>40.38441423170406</v>
+        <v>44.44731251339184</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>20.51032187739574</v>
+        <v>15.04700803777743</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.40780291198057</v>
+        <v>0.5944984271295312</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.2114490852073816</v>
+        <v>-0.334065529109323</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6667</v>
+        <v>6581</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>223.7525212855208</v>
+        <v>232.4922194540182</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>244</v>
+        <v>107</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>38.33373012687787</v>
+        <v>46.37175414619171</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>17.50043244615813</v>
+        <v>8.967333247108776</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.4884568224574405</v>
+        <v>1.388950364695412</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-2.198895149522224</v>
+        <v>0.0336541127624466</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6657</v>
+        <v>6558</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>華安</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>210.414511512619</v>
+        <v>226.1876616354878</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>35.85</v>
+        <v>27.7</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>49.52668107915056</v>
+        <v>40.38441423170406</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.14634449016008</v>
+        <v>20.51032187739574</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.947797389019744</v>
+        <v>0.40780291198057</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.1269125498667427</v>
+        <v>-0.2114490852073816</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6550</v>
+        <v>6667</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>北極星藥業-KY</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>201.0584502894279</v>
+        <v>223.7525212855208</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>12.05</v>
+        <v>244</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>36.88455952844517</v>
+        <v>38.33373012687787</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>21.22405142359455</v>
+        <v>17.50043244615813</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.371902735306184</v>
+        <v>0.4884568224574405</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0207545651756339</v>
+        <v>-2.198895149522224</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6512</v>
+        <v>6657</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>啟發電</t>
+          <t>華安</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>192.1332432134516</v>
+        <v>210.414511512619</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>20.2</v>
+        <v>35.85</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>52.55302233999326</v>
+        <v>49.52668107915056</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>10.24887024395368</v>
+        <v>18.14634449016008</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1.418828382589844</v>
+        <v>0.947797389019744</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.5437001671753194</v>
+        <v>0.1269125498667427</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6589</v>
+        <v>6550</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>台康生技</t>
+          <t>北極星藥業-KY</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>191.7272249901937</v>
+        <v>201.0584502894279</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>46.6</v>
+        <v>12.05</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>49.05217577728614</v>
+        <v>36.88455952844517</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>19.30092838661257</v>
+        <v>21.22405142359455</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.3855547915788709</v>
+        <v>1.371902735306184</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.4695191175505411</v>
+        <v>-0.0207545651756339</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6803</v>
+        <v>6512</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>啟發電</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>189.8327978566766</v>
+        <v>192.1332432134516</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>270</v>
+        <v>20.2</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>32.83238183743524</v>
+        <v>52.55302233999326</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>46.85658763603835</v>
+        <v>10.24887024395368</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.428992143931411</v>
+        <v>1.418828382589844</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.6941071664503125</v>
+        <v>0.5437001671753194</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6781</v>
+        <v>6589</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>台康生技</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>185.1338074577687</v>
+        <v>191.7272249901937</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>1005</v>
+        <v>46.6</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>40.14939387604348</v>
+        <v>49.05217577728614</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>19.15515790059528</v>
+        <v>19.30092838661257</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.5720916551334638</v>
+        <v>0.3855547915788709</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-20.20896154203329</v>
+        <v>-0.4695191175505411</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6823</v>
+        <v>6803</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>濾能</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>177.3161475549865</v>
+        <v>189.8327978566766</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>61.8</v>
+        <v>270</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>36.64328358637933</v>
+        <v>32.83238183743524</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.62094289083427</v>
+        <v>46.85658763603835</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4228745727291835</v>
+        <v>0.428992143931411</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.4547060388026513</v>
+        <v>-0.6941071664503125</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6591</v>
+        <v>6781</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>175.9670313927867</v>
+        <v>185.1338074577687</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>45</v>
+        <v>1005</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>29.75210981571462</v>
+        <v>40.14939387604348</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>40.14539797979163</v>
+        <v>19.15515790059528</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.5258437790505893</v>
+        <v>0.5720916551334638</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.6158581498897937</v>
+        <v>-20.20896154203329</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6597</v>
+        <v>6823</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>濾能</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>160.9901750648653</v>
+        <v>177.3161475549865</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>59.1</v>
+        <v>61.8</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.44094323170921</v>
+        <v>36.64328358637933</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>10.0164050583843</v>
+        <v>16.62094289083427</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.8392981513958933</v>
+        <v>0.4228745727291835</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.3354103379162447</v>
+        <v>-0.4547060388026513</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6720</v>
+        <v>6591</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>148.3621020159132</v>
+        <v>175.9670313927867</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>136</v>
+        <v>45</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>39.10586223742065</v>
+        <v>29.75210981571462</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>22.26133745318492</v>
+        <v>40.14539797979163</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.4741817506886413</v>
+        <v>0.5258437790505893</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.004660514335987</v>
+        <v>-0.6158581498897937</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6516,21 +6516,21 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6592</v>
+        <v>6597</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>147.6507295358981</v>
+        <v>160.9901750648653</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>60.5</v>
+        <v>59.1</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>44.97449336491166</v>
+        <v>47.44094323170921</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>17.87288010398461</v>
+        <v>10.0164050583843</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.2962110087309004</v>
+        <v>0.8392981513958933</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.029710391338079</v>
+        <v>0.3354103379162447</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6552</v>
+        <v>6720</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>144.606685233064</v>
+        <v>148.3621020159132</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>25.95</v>
+        <v>136</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>36.89536262654456</v>
+        <v>39.10586223742065</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>17.26177265723186</v>
+        <v>22.26133745318492</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6042242527660823</v>
+        <v>0.4741817506886413</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.4134479639708939</v>
+        <v>-0.004660514335987</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6668</v>
+        <v>6592</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>144.1698281199486</v>
+        <v>147.6507295358981</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>34.1</v>
+        <v>60.5</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>33.34710273351651</v>
+        <v>44.97449336491166</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>19.68658386128234</v>
+        <v>17.87288010398461</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.5066141891213359</v>
+        <v>0.2962110087309004</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.51223071075398</v>
+        <v>0.029710391338079</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6708</v>
+        <v>6552</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>144.1444560545653</v>
+        <v>144.606685233064</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>37.8</v>
+        <v>25.95</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>41.63074177028504</v>
+        <v>36.89536262654456</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>14.15928101429509</v>
+        <v>17.26177265723186</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.4663664634134542</v>
+        <v>0.6042242527660823</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1970303961524293</v>
+        <v>-0.4134479639708939</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6541</v>
+        <v>6668</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>136.4304936487662</v>
+        <v>144.1698281199486</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>40</v>
+        <v>34.1</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>48.62689998080948</v>
+        <v>33.34710273351651</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>12.68773976524556</v>
+        <v>19.68658386128234</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.7026750848310708</v>
+        <v>0.5066141891213359</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.1130532541452615</v>
+        <v>-0.51223071075398</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6781,21 +6781,21 @@
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6796</v>
+        <v>6708</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>晉弘</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>133.1780497829884</v>
+        <v>144.1444560545653</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>59.4</v>
+        <v>37.8</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,16 +6806,16 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>51.49405560650849</v>
+        <v>41.63074177028504</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.91907071991184</v>
+        <v>14.15928101429509</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>1.052216219816551</v>
+        <v>0.4663664634134542</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.2411383286367556</v>
+        <v>-0.1970303961524293</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6614</v>
+        <v>6541</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>105.8066736933022</v>
+        <v>136.4304936487662</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>38.35</v>
+        <v>40</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>36.34800780269328</v>
+        <v>48.62689998080948</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>16.91126571138404</v>
+        <v>12.68773976524556</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.8759519964846997</v>
+        <v>0.7026750848310708</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.1833110751191367</v>
+        <v>-0.1130532541452615</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6887,21 +6887,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6625</v>
+        <v>6796</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>晉弘</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>101.6062828865017</v>
+        <v>133.1780497829884</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>75.09999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>37.3222258253783</v>
+        <v>51.49405560650849</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>19.46301772243142</v>
+        <v>15.91907071991184</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.7429317190838437</v>
+        <v>1.052216219816551</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.5784504224020135</v>
+        <v>0.2411383286367556</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,18 +6940,18 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6771</v>
+        <v>6614</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>83.54593019514562</v>
+        <v>105.8066736933022</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>38.35</v>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>36.81214425074619</v>
+        <v>36.34800780269328</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>14.86707414271595</v>
+        <v>16.91126571138404</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.8825625055040069</v>
+        <v>0.8759519964846997</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.008501817322677199</v>
+        <v>-0.1833110751191367</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -6993,21 +6993,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6674</v>
+        <v>6625</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>必應</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>68.48638419815464</v>
+        <v>101.6062828865017</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>16.2</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>41.0087533811563</v>
+        <v>37.3222258253783</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>18.40436529929937</v>
+        <v>19.46301772243142</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.8792017784813073</v>
+        <v>0.7429317190838437</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.0346558685920534</v>
+        <v>-0.5784504224020135</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,52 +7046,158 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
+        <v>6771</v>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>平和環保-創</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>83.54593019514562</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>38.35</v>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H125" s="2" t="n">
+        <v>36.81214425074619</v>
+      </c>
+      <c r="I125" s="2" t="n">
+        <v>14.86707414271595</v>
+      </c>
+      <c r="J125" s="2" t="n">
+        <v>0.8825625055040069</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N125" s="2" t="n">
+        <v>0.008501817322677199</v>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>6674</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>鋐寶科技</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>68.48638419815464</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>41.0087533811563</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>18.40436529929937</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.8792017784813073</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>-0.0346558685920534</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
         <v>6692</v>
       </c>
-      <c r="B125" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>進能服</t>
         </is>
       </c>
-      <c r="C125" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D125" s="2" t="n">
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>60.93603940883918</v>
       </c>
-      <c r="E125" s="2" t="n">
+      <c r="E127" s="2" t="n">
         <v>23.95</v>
       </c>
-      <c r="F125" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="G125" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H125" s="2" t="n">
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>42.20994507252375</v>
       </c>
-      <c r="I125" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>14.24159462002697</v>
       </c>
-      <c r="J125" s="2" t="n">
+      <c r="J127" s="2" t="n">
         <v>0.4509314401514782</v>
       </c>
-      <c r="K125" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L125" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M125" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N125" s="2" t="n">
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
         <v>-0.0831965975328775</v>
       </c>
-      <c r="O125" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>